<commit_message>
Ajout de modifications dans le dictionnaire des données
</commit_message>
<xml_diff>
--- a/03_Analyse/dictionnaire_donnes.xlsx.xlsx
+++ b/03_Analyse/dictionnaire_donnes.xlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://genmills-my.sharepoint.com/personal/joffray_dealberto_genmills_com/Documents/Desktop/Dossier Perso/Github/IBM_HR_BA_Mission/03_Analyse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="319" documentId="11_F25DC773A252ABDACC10482BD9DC6EA45ADE58F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8AEBE48-163C-4D1F-9838-380CD014FC64}"/>
+  <xr:revisionPtr revIDLastSave="320" documentId="11_F25DC773A252ABDACC10482BD9DC6EA45ADE58F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CA6D76F-56F4-4741-BB5F-5234D12DF2DB}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1009,7 +1009,7 @@
         <v>75</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>76</v>
+        <v>121</v>
       </c>
       <c r="E12" t="s">
         <v>11</v>

</xml_diff>